<commit_message>
long format excel fixed, cleaned repo
</commit_message>
<xml_diff>
--- a/Input/urbs_intertemporal_master.xlsx
+++ b/Input/urbs_intertemporal_master.xlsx
@@ -54879,7 +54879,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>17304.86110833333</v>
+        <v>207658.3333</v>
       </c>
     </row>
     <row r="4">
@@ -54890,7 +54890,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>17304.86110833333</v>
+        <v>207658.3333</v>
       </c>
     </row>
     <row r="5">
@@ -54901,7 +54901,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>17304.86110833333</v>
+        <v>207658.3333</v>
       </c>
     </row>
     <row r="6">
@@ -54912,7 +54912,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>17304.86110833333</v>
+        <v>207658.3333</v>
       </c>
     </row>
     <row r="7">
@@ -54923,7 +54923,7 @@
         <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>17304.86110833333</v>
+        <v>207658.3333</v>
       </c>
     </row>
     <row r="8">
@@ -54934,7 +54934,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>17304.86110833333</v>
+        <v>207658.3333</v>
       </c>
     </row>
     <row r="9">
@@ -54945,7 +54945,7 @@
         <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>17304.86110833333</v>
+        <v>207658.3333</v>
       </c>
     </row>
     <row r="10">
@@ -54956,7 +54956,7 @@
         <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>17304.86110833333</v>
+        <v>207658.3333</v>
       </c>
     </row>
     <row r="11">
@@ -54967,7 +54967,7 @@
         <v>9</v>
       </c>
       <c r="C11" t="n">
-        <v>17304.86110833333</v>
+        <v>207658.3333</v>
       </c>
     </row>
     <row r="12">
@@ -54978,7 +54978,7 @@
         <v>10</v>
       </c>
       <c r="C12" t="n">
-        <v>17304.86110833333</v>
+        <v>207658.3333</v>
       </c>
     </row>
     <row r="13">
@@ -54989,7 +54989,7 @@
         <v>11</v>
       </c>
       <c r="C13" t="n">
-        <v>17304.86110833333</v>
+        <v>207658.3333</v>
       </c>
     </row>
     <row r="14">
@@ -55000,7 +55000,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>17304.86110833333</v>
+        <v>207658.3333</v>
       </c>
     </row>
     <row r="15">
@@ -55022,7 +55022,7 @@
         <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>17965.66823333333</v>
+        <v>215588.0188</v>
       </c>
     </row>
     <row r="17">
@@ -55033,7 +55033,7 @@
         <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>17965.66823333333</v>
+        <v>215588.0188</v>
       </c>
     </row>
     <row r="18">
@@ -55044,7 +55044,7 @@
         <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>17965.66823333333</v>
+        <v>215588.0188</v>
       </c>
     </row>
     <row r="19">
@@ -55055,7 +55055,7 @@
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>17965.66823333333</v>
+        <v>215588.0188</v>
       </c>
     </row>
     <row r="20">
@@ -55066,7 +55066,7 @@
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>17965.66823333333</v>
+        <v>215588.0188</v>
       </c>
     </row>
     <row r="21">
@@ -55077,7 +55077,7 @@
         <v>6</v>
       </c>
       <c r="C21" t="n">
-        <v>17965.66823333333</v>
+        <v>215588.0188</v>
       </c>
     </row>
     <row r="22">
@@ -55088,7 +55088,7 @@
         <v>7</v>
       </c>
       <c r="C22" t="n">
-        <v>17965.66823333333</v>
+        <v>215588.0188</v>
       </c>
     </row>
     <row r="23">
@@ -55099,7 +55099,7 @@
         <v>8</v>
       </c>
       <c r="C23" t="n">
-        <v>17965.66823333333</v>
+        <v>215588.0188</v>
       </c>
     </row>
     <row r="24">
@@ -55110,7 +55110,7 @@
         <v>9</v>
       </c>
       <c r="C24" t="n">
-        <v>17965.66823333333</v>
+        <v>215588.0188</v>
       </c>
     </row>
     <row r="25">
@@ -55121,7 +55121,7 @@
         <v>10</v>
       </c>
       <c r="C25" t="n">
-        <v>17965.66823333333</v>
+        <v>215588.0188</v>
       </c>
     </row>
     <row r="26">
@@ -55132,7 +55132,7 @@
         <v>11</v>
       </c>
       <c r="C26" t="n">
-        <v>17965.66823333333</v>
+        <v>215588.0188</v>
       </c>
     </row>
     <row r="27">
@@ -55143,7 +55143,7 @@
         <v>12</v>
       </c>
       <c r="C27" t="n">
-        <v>17965.66823333333</v>
+        <v>215588.0188</v>
       </c>
     </row>
     <row r="28">
@@ -55165,7 +55165,7 @@
         <v>1</v>
       </c>
       <c r="C29" t="n">
-        <v>18626.47535</v>
+        <v>223517.7042</v>
       </c>
     </row>
     <row r="30">
@@ -55176,7 +55176,7 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>18626.47535</v>
+        <v>223517.7042</v>
       </c>
     </row>
     <row r="31">
@@ -55187,7 +55187,7 @@
         <v>3</v>
       </c>
       <c r="C31" t="n">
-        <v>18626.47535</v>
+        <v>223517.7042</v>
       </c>
     </row>
     <row r="32">
@@ -55198,7 +55198,7 @@
         <v>4</v>
       </c>
       <c r="C32" t="n">
-        <v>18626.47535</v>
+        <v>223517.7042</v>
       </c>
     </row>
     <row r="33">
@@ -55209,7 +55209,7 @@
         <v>5</v>
       </c>
       <c r="C33" t="n">
-        <v>18626.47535</v>
+        <v>223517.7042</v>
       </c>
     </row>
     <row r="34">
@@ -55220,7 +55220,7 @@
         <v>6</v>
       </c>
       <c r="C34" t="n">
-        <v>18626.47535</v>
+        <v>223517.7042</v>
       </c>
     </row>
     <row r="35">
@@ -55231,7 +55231,7 @@
         <v>7</v>
       </c>
       <c r="C35" t="n">
-        <v>18626.47535</v>
+        <v>223517.7042</v>
       </c>
     </row>
     <row r="36">
@@ -55242,7 +55242,7 @@
         <v>8</v>
       </c>
       <c r="C36" t="n">
-        <v>18626.47535</v>
+        <v>223517.7042</v>
       </c>
     </row>
     <row r="37">
@@ -55253,7 +55253,7 @@
         <v>9</v>
       </c>
       <c r="C37" t="n">
-        <v>18626.47535</v>
+        <v>223517.7042</v>
       </c>
     </row>
     <row r="38">
@@ -55264,7 +55264,7 @@
         <v>10</v>
       </c>
       <c r="C38" t="n">
-        <v>18626.47535</v>
+        <v>223517.7042</v>
       </c>
     </row>
     <row r="39">
@@ -55275,7 +55275,7 @@
         <v>11</v>
       </c>
       <c r="C39" t="n">
-        <v>18626.47535</v>
+        <v>223517.7042</v>
       </c>
     </row>
     <row r="40">
@@ -55286,7 +55286,7 @@
         <v>12</v>
       </c>
       <c r="C40" t="n">
-        <v>18626.47535</v>
+        <v>223517.7042</v>
       </c>
     </row>
     <row r="41">
@@ -55308,7 +55308,7 @@
         <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>19287.28246666667</v>
+        <v>231447.3896</v>
       </c>
     </row>
     <row r="43">
@@ -55319,7 +55319,7 @@
         <v>2</v>
       </c>
       <c r="C43" t="n">
-        <v>19287.28246666667</v>
+        <v>231447.3896</v>
       </c>
     </row>
     <row r="44">
@@ -55330,7 +55330,7 @@
         <v>3</v>
       </c>
       <c r="C44" t="n">
-        <v>19287.28246666667</v>
+        <v>231447.3896</v>
       </c>
     </row>
     <row r="45">
@@ -55341,7 +55341,7 @@
         <v>4</v>
       </c>
       <c r="C45" t="n">
-        <v>19287.28246666667</v>
+        <v>231447.3896</v>
       </c>
     </row>
     <row r="46">
@@ -55352,7 +55352,7 @@
         <v>5</v>
       </c>
       <c r="C46" t="n">
-        <v>19287.28246666667</v>
+        <v>231447.3896</v>
       </c>
     </row>
     <row r="47">
@@ -55363,7 +55363,7 @@
         <v>6</v>
       </c>
       <c r="C47" t="n">
-        <v>19287.28246666667</v>
+        <v>231447.3896</v>
       </c>
     </row>
     <row r="48">
@@ -55374,7 +55374,7 @@
         <v>7</v>
       </c>
       <c r="C48" t="n">
-        <v>19287.28246666667</v>
+        <v>231447.3896</v>
       </c>
     </row>
     <row r="49">
@@ -55385,7 +55385,7 @@
         <v>8</v>
       </c>
       <c r="C49" t="n">
-        <v>19287.28246666667</v>
+        <v>231447.3896</v>
       </c>
     </row>
     <row r="50">
@@ -55396,7 +55396,7 @@
         <v>9</v>
       </c>
       <c r="C50" t="n">
-        <v>19287.28246666667</v>
+        <v>231447.3896</v>
       </c>
     </row>
     <row r="51">
@@ -55407,7 +55407,7 @@
         <v>10</v>
       </c>
       <c r="C51" t="n">
-        <v>19287.28246666667</v>
+        <v>231447.3896</v>
       </c>
     </row>
     <row r="52">
@@ -55418,7 +55418,7 @@
         <v>11</v>
       </c>
       <c r="C52" t="n">
-        <v>19287.28246666667</v>
+        <v>231447.3896</v>
       </c>
     </row>
     <row r="53">
@@ -55429,7 +55429,7 @@
         <v>12</v>
       </c>
       <c r="C53" t="n">
-        <v>19287.28246666667</v>
+        <v>231447.3896</v>
       </c>
     </row>
     <row r="54">
@@ -55451,7 +55451,7 @@
         <v>1</v>
       </c>
       <c r="C55" t="n">
-        <v>19948.08959166667</v>
+        <v>239377.0751</v>
       </c>
     </row>
     <row r="56">
@@ -55462,7 +55462,7 @@
         <v>2</v>
       </c>
       <c r="C56" t="n">
-        <v>19948.08959166667</v>
+        <v>239377.0751</v>
       </c>
     </row>
     <row r="57">
@@ -55473,7 +55473,7 @@
         <v>3</v>
       </c>
       <c r="C57" t="n">
-        <v>19948.08959166667</v>
+        <v>239377.0751</v>
       </c>
     </row>
     <row r="58">
@@ -55484,7 +55484,7 @@
         <v>4</v>
       </c>
       <c r="C58" t="n">
-        <v>19948.08959166667</v>
+        <v>239377.0751</v>
       </c>
     </row>
     <row r="59">
@@ -55495,7 +55495,7 @@
         <v>5</v>
       </c>
       <c r="C59" t="n">
-        <v>19948.08959166667</v>
+        <v>239377.0751</v>
       </c>
     </row>
     <row r="60">
@@ -55506,7 +55506,7 @@
         <v>6</v>
       </c>
       <c r="C60" t="n">
-        <v>19948.08959166667</v>
+        <v>239377.0751</v>
       </c>
     </row>
     <row r="61">
@@ -55517,7 +55517,7 @@
         <v>7</v>
       </c>
       <c r="C61" t="n">
-        <v>19948.08959166667</v>
+        <v>239377.0751</v>
       </c>
     </row>
     <row r="62">
@@ -55528,7 +55528,7 @@
         <v>8</v>
       </c>
       <c r="C62" t="n">
-        <v>19948.08959166667</v>
+        <v>239377.0751</v>
       </c>
     </row>
     <row r="63">
@@ -55539,7 +55539,7 @@
         <v>9</v>
       </c>
       <c r="C63" t="n">
-        <v>19948.08959166667</v>
+        <v>239377.0751</v>
       </c>
     </row>
     <row r="64">
@@ -55550,7 +55550,7 @@
         <v>10</v>
       </c>
       <c r="C64" t="n">
-        <v>19948.08959166667</v>
+        <v>239377.0751</v>
       </c>
     </row>
     <row r="65">
@@ -55561,7 +55561,7 @@
         <v>11</v>
       </c>
       <c r="C65" t="n">
-        <v>19948.08959166667</v>
+        <v>239377.0751</v>
       </c>
     </row>
     <row r="66">
@@ -55572,7 +55572,7 @@
         <v>12</v>
       </c>
       <c r="C66" t="n">
-        <v>19948.08959166667</v>
+        <v>239377.0751</v>
       </c>
     </row>
     <row r="67">
@@ -55594,7 +55594,7 @@
         <v>1</v>
       </c>
       <c r="C68" t="n">
-        <v>20608.89670833333</v>
+        <v>247306.7605</v>
       </c>
     </row>
     <row r="69">
@@ -55605,7 +55605,7 @@
         <v>2</v>
       </c>
       <c r="C69" t="n">
-        <v>20608.89670833333</v>
+        <v>247306.7605</v>
       </c>
     </row>
     <row r="70">
@@ -55616,7 +55616,7 @@
         <v>3</v>
       </c>
       <c r="C70" t="n">
-        <v>20608.89670833333</v>
+        <v>247306.7605</v>
       </c>
     </row>
     <row r="71">
@@ -55627,7 +55627,7 @@
         <v>4</v>
       </c>
       <c r="C71" t="n">
-        <v>20608.89670833333</v>
+        <v>247306.7605</v>
       </c>
     </row>
     <row r="72">
@@ -55638,7 +55638,7 @@
         <v>5</v>
       </c>
       <c r="C72" t="n">
-        <v>20608.89670833333</v>
+        <v>247306.7605</v>
       </c>
     </row>
     <row r="73">
@@ -55649,7 +55649,7 @@
         <v>6</v>
       </c>
       <c r="C73" t="n">
-        <v>20608.89670833333</v>
+        <v>247306.7605</v>
       </c>
     </row>
     <row r="74">
@@ -55660,7 +55660,7 @@
         <v>7</v>
       </c>
       <c r="C74" t="n">
-        <v>20608.89670833333</v>
+        <v>247306.7605</v>
       </c>
     </row>
     <row r="75">
@@ -55671,7 +55671,7 @@
         <v>8</v>
       </c>
       <c r="C75" t="n">
-        <v>20608.89670833333</v>
+        <v>247306.7605</v>
       </c>
     </row>
     <row r="76">
@@ -55682,7 +55682,7 @@
         <v>9</v>
       </c>
       <c r="C76" t="n">
-        <v>20608.89670833333</v>
+        <v>247306.7605</v>
       </c>
     </row>
     <row r="77">
@@ -55693,7 +55693,7 @@
         <v>10</v>
       </c>
       <c r="C77" t="n">
-        <v>20608.89670833333</v>
+        <v>247306.7605</v>
       </c>
     </row>
     <row r="78">
@@ -55704,7 +55704,7 @@
         <v>11</v>
       </c>
       <c r="C78" t="n">
-        <v>20608.89670833333</v>
+        <v>247306.7605</v>
       </c>
     </row>
     <row r="79">
@@ -55715,7 +55715,7 @@
         <v>12</v>
       </c>
       <c r="C79" t="n">
-        <v>20608.89670833333</v>
+        <v>247306.7605</v>
       </c>
     </row>
     <row r="80">
@@ -55737,7 +55737,7 @@
         <v>1</v>
       </c>
       <c r="C81" t="n">
-        <v>21269.703825</v>
+        <v>255236.4459</v>
       </c>
     </row>
     <row r="82">
@@ -55748,7 +55748,7 @@
         <v>2</v>
       </c>
       <c r="C82" t="n">
-        <v>21269.703825</v>
+        <v>255236.4459</v>
       </c>
     </row>
     <row r="83">
@@ -55759,7 +55759,7 @@
         <v>3</v>
       </c>
       <c r="C83" t="n">
-        <v>21269.703825</v>
+        <v>255236.4459</v>
       </c>
     </row>
     <row r="84">
@@ -55770,7 +55770,7 @@
         <v>4</v>
       </c>
       <c r="C84" t="n">
-        <v>21269.703825</v>
+        <v>255236.4459</v>
       </c>
     </row>
     <row r="85">
@@ -55781,7 +55781,7 @@
         <v>5</v>
       </c>
       <c r="C85" t="n">
-        <v>21269.703825</v>
+        <v>255236.4459</v>
       </c>
     </row>
     <row r="86">
@@ -55792,7 +55792,7 @@
         <v>6</v>
       </c>
       <c r="C86" t="n">
-        <v>21269.703825</v>
+        <v>255236.4459</v>
       </c>
     </row>
     <row r="87">
@@ -55803,7 +55803,7 @@
         <v>7</v>
       </c>
       <c r="C87" t="n">
-        <v>21269.703825</v>
+        <v>255236.4459</v>
       </c>
     </row>
     <row r="88">
@@ -55814,7 +55814,7 @@
         <v>8</v>
       </c>
       <c r="C88" t="n">
-        <v>21269.703825</v>
+        <v>255236.4459</v>
       </c>
     </row>
     <row r="89">
@@ -55825,7 +55825,7 @@
         <v>9</v>
       </c>
       <c r="C89" t="n">
-        <v>21269.703825</v>
+        <v>255236.4459</v>
       </c>
     </row>
     <row r="90">
@@ -55836,7 +55836,7 @@
         <v>10</v>
       </c>
       <c r="C90" t="n">
-        <v>21269.703825</v>
+        <v>255236.4459</v>
       </c>
     </row>
     <row r="91">
@@ -55847,7 +55847,7 @@
         <v>11</v>
       </c>
       <c r="C91" t="n">
-        <v>21269.703825</v>
+        <v>255236.4459</v>
       </c>
     </row>
     <row r="92">
@@ -55858,7 +55858,7 @@
         <v>12</v>
       </c>
       <c r="C92" t="n">
-        <v>21269.703825</v>
+        <v>255236.4459</v>
       </c>
     </row>
     <row r="93">
@@ -55880,7 +55880,7 @@
         <v>1</v>
       </c>
       <c r="C94" t="n">
-        <v>21674.80408333333</v>
+        <v>260097.649</v>
       </c>
     </row>
     <row r="95">
@@ -55891,7 +55891,7 @@
         <v>2</v>
       </c>
       <c r="C95" t="n">
-        <v>21674.80408333333</v>
+        <v>260097.649</v>
       </c>
     </row>
     <row r="96">
@@ -55902,7 +55902,7 @@
         <v>3</v>
       </c>
       <c r="C96" t="n">
-        <v>21674.80408333333</v>
+        <v>260097.649</v>
       </c>
     </row>
     <row r="97">
@@ -55913,7 +55913,7 @@
         <v>4</v>
       </c>
       <c r="C97" t="n">
-        <v>21674.80408333333</v>
+        <v>260097.649</v>
       </c>
     </row>
     <row r="98">
@@ -55924,7 +55924,7 @@
         <v>5</v>
       </c>
       <c r="C98" t="n">
-        <v>21674.80408333333</v>
+        <v>260097.649</v>
       </c>
     </row>
     <row r="99">
@@ -55935,7 +55935,7 @@
         <v>6</v>
       </c>
       <c r="C99" t="n">
-        <v>21674.80408333333</v>
+        <v>260097.649</v>
       </c>
     </row>
     <row r="100">
@@ -55946,7 +55946,7 @@
         <v>7</v>
       </c>
       <c r="C100" t="n">
-        <v>21674.80408333333</v>
+        <v>260097.649</v>
       </c>
     </row>
     <row r="101">
@@ -55957,7 +55957,7 @@
         <v>8</v>
       </c>
       <c r="C101" t="n">
-        <v>21674.80408333333</v>
+        <v>260097.649</v>
       </c>
     </row>
     <row r="102">
@@ -55968,7 +55968,7 @@
         <v>9</v>
       </c>
       <c r="C102" t="n">
-        <v>21674.80408333333</v>
+        <v>260097.649</v>
       </c>
     </row>
     <row r="103">
@@ -55979,7 +55979,7 @@
         <v>10</v>
       </c>
       <c r="C103" t="n">
-        <v>21674.80408333333</v>
+        <v>260097.649</v>
       </c>
     </row>
     <row r="104">
@@ -55990,7 +55990,7 @@
         <v>11</v>
       </c>
       <c r="C104" t="n">
-        <v>21674.80408333333</v>
+        <v>260097.649</v>
       </c>
     </row>
     <row r="105">
@@ -56001,7 +56001,7 @@
         <v>12</v>
       </c>
       <c r="C105" t="n">
-        <v>21674.80408333333</v>
+        <v>260097.649</v>
       </c>
     </row>
     <row r="106">
@@ -56023,7 +56023,7 @@
         <v>1</v>
       </c>
       <c r="C107" t="n">
-        <v>22079.90434166667</v>
+        <v>264958.8521</v>
       </c>
     </row>
     <row r="108">
@@ -56034,7 +56034,7 @@
         <v>2</v>
       </c>
       <c r="C108" t="n">
-        <v>22079.90434166667</v>
+        <v>264958.8521</v>
       </c>
     </row>
     <row r="109">
@@ -56045,7 +56045,7 @@
         <v>3</v>
       </c>
       <c r="C109" t="n">
-        <v>22079.90434166667</v>
+        <v>264958.8521</v>
       </c>
     </row>
     <row r="110">
@@ -56056,7 +56056,7 @@
         <v>4</v>
       </c>
       <c r="C110" t="n">
-        <v>22079.90434166667</v>
+        <v>264958.8521</v>
       </c>
     </row>
     <row r="111">
@@ -56067,7 +56067,7 @@
         <v>5</v>
       </c>
       <c r="C111" t="n">
-        <v>22079.90434166667</v>
+        <v>264958.8521</v>
       </c>
     </row>
     <row r="112">
@@ -56078,7 +56078,7 @@
         <v>6</v>
       </c>
       <c r="C112" t="n">
-        <v>22079.90434166667</v>
+        <v>264958.8521</v>
       </c>
     </row>
     <row r="113">
@@ -56089,7 +56089,7 @@
         <v>7</v>
       </c>
       <c r="C113" t="n">
-        <v>22079.90434166667</v>
+        <v>264958.8521</v>
       </c>
     </row>
     <row r="114">
@@ -56100,7 +56100,7 @@
         <v>8</v>
       </c>
       <c r="C114" t="n">
-        <v>22079.90434166667</v>
+        <v>264958.8521</v>
       </c>
     </row>
     <row r="115">
@@ -56111,7 +56111,7 @@
         <v>9</v>
       </c>
       <c r="C115" t="n">
-        <v>22079.90434166667</v>
+        <v>264958.8521</v>
       </c>
     </row>
     <row r="116">
@@ -56122,7 +56122,7 @@
         <v>10</v>
       </c>
       <c r="C116" t="n">
-        <v>22079.90434166667</v>
+        <v>264958.8521</v>
       </c>
     </row>
     <row r="117">
@@ -56133,7 +56133,7 @@
         <v>11</v>
       </c>
       <c r="C117" t="n">
-        <v>22079.90434166667</v>
+        <v>264958.8521</v>
       </c>
     </row>
     <row r="118">
@@ -56144,7 +56144,7 @@
         <v>12</v>
       </c>
       <c r="C118" t="n">
-        <v>22079.90434166667</v>
+        <v>264958.8521</v>
       </c>
     </row>
     <row r="119">
@@ -56166,7 +56166,7 @@
         <v>1</v>
       </c>
       <c r="C120" t="n">
-        <v>22485.00460833333</v>
+        <v>269820.0553</v>
       </c>
     </row>
     <row r="121">
@@ -56177,7 +56177,7 @@
         <v>2</v>
       </c>
       <c r="C121" t="n">
-        <v>22485.00460833333</v>
+        <v>269820.0553</v>
       </c>
     </row>
     <row r="122">
@@ -56188,7 +56188,7 @@
         <v>3</v>
       </c>
       <c r="C122" t="n">
-        <v>22485.00460833333</v>
+        <v>269820.0553</v>
       </c>
     </row>
     <row r="123">
@@ -56199,7 +56199,7 @@
         <v>4</v>
       </c>
       <c r="C123" t="n">
-        <v>22485.00460833333</v>
+        <v>269820.0553</v>
       </c>
     </row>
     <row r="124">
@@ -56210,7 +56210,7 @@
         <v>5</v>
       </c>
       <c r="C124" t="n">
-        <v>22485.00460833333</v>
+        <v>269820.0553</v>
       </c>
     </row>
     <row r="125">
@@ -56221,7 +56221,7 @@
         <v>6</v>
       </c>
       <c r="C125" t="n">
-        <v>22485.00460833333</v>
+        <v>269820.0553</v>
       </c>
     </row>
     <row r="126">
@@ -56232,7 +56232,7 @@
         <v>7</v>
       </c>
       <c r="C126" t="n">
-        <v>22485.00460833333</v>
+        <v>269820.0553</v>
       </c>
     </row>
     <row r="127">
@@ -56243,7 +56243,7 @@
         <v>8</v>
       </c>
       <c r="C127" t="n">
-        <v>22485.00460833333</v>
+        <v>269820.0553</v>
       </c>
     </row>
     <row r="128">
@@ -56254,7 +56254,7 @@
         <v>9</v>
       </c>
       <c r="C128" t="n">
-        <v>22485.00460833333</v>
+        <v>269820.0553</v>
       </c>
     </row>
     <row r="129">
@@ -56265,7 +56265,7 @@
         <v>10</v>
       </c>
       <c r="C129" t="n">
-        <v>22485.00460833333</v>
+        <v>269820.0553</v>
       </c>
     </row>
     <row r="130">
@@ -56276,7 +56276,7 @@
         <v>11</v>
       </c>
       <c r="C130" t="n">
-        <v>22485.00460833333</v>
+        <v>269820.0553</v>
       </c>
     </row>
     <row r="131">
@@ -56287,7 +56287,7 @@
         <v>12</v>
       </c>
       <c r="C131" t="n">
-        <v>22485.00460833333</v>
+        <v>269820.0553</v>
       </c>
     </row>
     <row r="132">
@@ -56309,7 +56309,7 @@
         <v>1</v>
       </c>
       <c r="C133" t="n">
-        <v>22890.10485833334</v>
+        <v>274681.2583</v>
       </c>
     </row>
     <row r="134">
@@ -56320,7 +56320,7 @@
         <v>2</v>
       </c>
       <c r="C134" t="n">
-        <v>22890.10485833334</v>
+        <v>274681.2583</v>
       </c>
     </row>
     <row r="135">
@@ -56331,7 +56331,7 @@
         <v>3</v>
       </c>
       <c r="C135" t="n">
-        <v>22890.10485833334</v>
+        <v>274681.2583</v>
       </c>
     </row>
     <row r="136">
@@ -56342,7 +56342,7 @@
         <v>4</v>
       </c>
       <c r="C136" t="n">
-        <v>22890.10485833334</v>
+        <v>274681.2583</v>
       </c>
     </row>
     <row r="137">
@@ -56353,7 +56353,7 @@
         <v>5</v>
       </c>
       <c r="C137" t="n">
-        <v>22890.10485833334</v>
+        <v>274681.2583</v>
       </c>
     </row>
     <row r="138">
@@ -56364,7 +56364,7 @@
         <v>6</v>
       </c>
       <c r="C138" t="n">
-        <v>22890.10485833334</v>
+        <v>274681.2583</v>
       </c>
     </row>
     <row r="139">
@@ -56375,7 +56375,7 @@
         <v>7</v>
       </c>
       <c r="C139" t="n">
-        <v>22890.10485833334</v>
+        <v>274681.2583</v>
       </c>
     </row>
     <row r="140">
@@ -56386,7 +56386,7 @@
         <v>8</v>
       </c>
       <c r="C140" t="n">
-        <v>22890.10485833334</v>
+        <v>274681.2583</v>
       </c>
     </row>
     <row r="141">
@@ -56397,7 +56397,7 @@
         <v>9</v>
       </c>
       <c r="C141" t="n">
-        <v>22890.10485833334</v>
+        <v>274681.2583</v>
       </c>
     </row>
     <row r="142">
@@ -56408,7 +56408,7 @@
         <v>10</v>
       </c>
       <c r="C142" t="n">
-        <v>22890.10485833334</v>
+        <v>274681.2583</v>
       </c>
     </row>
     <row r="143">
@@ -56419,7 +56419,7 @@
         <v>11</v>
       </c>
       <c r="C143" t="n">
-        <v>22890.10485833334</v>
+        <v>274681.2583</v>
       </c>
     </row>
     <row r="144">
@@ -56430,7 +56430,7 @@
         <v>12</v>
       </c>
       <c r="C144" t="n">
-        <v>22890.10485833334</v>
+        <v>274681.2583</v>
       </c>
     </row>
     <row r="145">
@@ -56452,7 +56452,7 @@
         <v>1</v>
       </c>
       <c r="C146" t="n">
-        <v>23295.205125</v>
+        <v>279542.4615</v>
       </c>
     </row>
     <row r="147">
@@ -56463,7 +56463,7 @@
         <v>2</v>
       </c>
       <c r="C147" t="n">
-        <v>23295.205125</v>
+        <v>279542.4615</v>
       </c>
     </row>
     <row r="148">
@@ -56474,7 +56474,7 @@
         <v>3</v>
       </c>
       <c r="C148" t="n">
-        <v>23295.205125</v>
+        <v>279542.4615</v>
       </c>
     </row>
     <row r="149">
@@ -56485,7 +56485,7 @@
         <v>4</v>
       </c>
       <c r="C149" t="n">
-        <v>23295.205125</v>
+        <v>279542.4615</v>
       </c>
     </row>
     <row r="150">
@@ -56496,7 +56496,7 @@
         <v>5</v>
       </c>
       <c r="C150" t="n">
-        <v>23295.205125</v>
+        <v>279542.4615</v>
       </c>
     </row>
     <row r="151">
@@ -56507,7 +56507,7 @@
         <v>6</v>
       </c>
       <c r="C151" t="n">
-        <v>23295.205125</v>
+        <v>279542.4615</v>
       </c>
     </row>
     <row r="152">
@@ -56518,7 +56518,7 @@
         <v>7</v>
       </c>
       <c r="C152" t="n">
-        <v>23295.205125</v>
+        <v>279542.4615</v>
       </c>
     </row>
     <row r="153">
@@ -56529,7 +56529,7 @@
         <v>8</v>
       </c>
       <c r="C153" t="n">
-        <v>23295.205125</v>
+        <v>279542.4615</v>
       </c>
     </row>
     <row r="154">
@@ -56540,7 +56540,7 @@
         <v>9</v>
       </c>
       <c r="C154" t="n">
-        <v>23295.205125</v>
+        <v>279542.4615</v>
       </c>
     </row>
     <row r="155">
@@ -56551,7 +56551,7 @@
         <v>10</v>
       </c>
       <c r="C155" t="n">
-        <v>23295.205125</v>
+        <v>279542.4615</v>
       </c>
     </row>
     <row r="156">
@@ -56562,7 +56562,7 @@
         <v>11</v>
       </c>
       <c r="C156" t="n">
-        <v>23295.205125</v>
+        <v>279542.4615</v>
       </c>
     </row>
     <row r="157">
@@ -56573,7 +56573,7 @@
         <v>12</v>
       </c>
       <c r="C157" t="n">
-        <v>23295.205125</v>
+        <v>279542.4615</v>
       </c>
     </row>
     <row r="158">
@@ -56595,7 +56595,7 @@
         <v>1</v>
       </c>
       <c r="C159" t="n">
-        <v>23700.30538333334</v>
+        <v>284403.6646</v>
       </c>
     </row>
     <row r="160">
@@ -56606,7 +56606,7 @@
         <v>2</v>
       </c>
       <c r="C160" t="n">
-        <v>23700.30538333334</v>
+        <v>284403.6646</v>
       </c>
     </row>
     <row r="161">
@@ -56617,7 +56617,7 @@
         <v>3</v>
       </c>
       <c r="C161" t="n">
-        <v>23700.30538333334</v>
+        <v>284403.6646</v>
       </c>
     </row>
     <row r="162">
@@ -56628,7 +56628,7 @@
         <v>4</v>
       </c>
       <c r="C162" t="n">
-        <v>23700.30538333334</v>
+        <v>284403.6646</v>
       </c>
     </row>
     <row r="163">
@@ -56639,7 +56639,7 @@
         <v>5</v>
       </c>
       <c r="C163" t="n">
-        <v>23700.30538333334</v>
+        <v>284403.6646</v>
       </c>
     </row>
     <row r="164">
@@ -56650,7 +56650,7 @@
         <v>6</v>
       </c>
       <c r="C164" t="n">
-        <v>23700.30538333334</v>
+        <v>284403.6646</v>
       </c>
     </row>
     <row r="165">
@@ -56661,7 +56661,7 @@
         <v>7</v>
       </c>
       <c r="C165" t="n">
-        <v>23700.30538333334</v>
+        <v>284403.6646</v>
       </c>
     </row>
     <row r="166">
@@ -56672,7 +56672,7 @@
         <v>8</v>
       </c>
       <c r="C166" t="n">
-        <v>23700.30538333334</v>
+        <v>284403.6646</v>
       </c>
     </row>
     <row r="167">
@@ -56683,7 +56683,7 @@
         <v>9</v>
       </c>
       <c r="C167" t="n">
-        <v>23700.30538333334</v>
+        <v>284403.6646</v>
       </c>
     </row>
     <row r="168">
@@ -56694,7 +56694,7 @@
         <v>10</v>
       </c>
       <c r="C168" t="n">
-        <v>23700.30538333334</v>
+        <v>284403.6646</v>
       </c>
     </row>
     <row r="169">
@@ -56705,7 +56705,7 @@
         <v>11</v>
       </c>
       <c r="C169" t="n">
-        <v>23700.30538333334</v>
+        <v>284403.6646</v>
       </c>
     </row>
     <row r="170">
@@ -56716,7 +56716,7 @@
         <v>12</v>
       </c>
       <c r="C170" t="n">
-        <v>23700.30538333334</v>
+        <v>284403.6646</v>
       </c>
     </row>
     <row r="171">
@@ -56738,7 +56738,7 @@
         <v>1</v>
       </c>
       <c r="C172" t="n">
-        <v>24105.40565</v>
+        <v>289264.8678</v>
       </c>
     </row>
     <row r="173">
@@ -56749,7 +56749,7 @@
         <v>2</v>
       </c>
       <c r="C173" t="n">
-        <v>24105.40565</v>
+        <v>289264.8678</v>
       </c>
     </row>
     <row r="174">
@@ -56760,7 +56760,7 @@
         <v>3</v>
       </c>
       <c r="C174" t="n">
-        <v>24105.40565</v>
+        <v>289264.8678</v>
       </c>
     </row>
     <row r="175">
@@ -56771,7 +56771,7 @@
         <v>4</v>
       </c>
       <c r="C175" t="n">
-        <v>24105.40565</v>
+        <v>289264.8678</v>
       </c>
     </row>
     <row r="176">
@@ -56782,7 +56782,7 @@
         <v>5</v>
       </c>
       <c r="C176" t="n">
-        <v>24105.40565</v>
+        <v>289264.8678</v>
       </c>
     </row>
     <row r="177">
@@ -56793,7 +56793,7 @@
         <v>6</v>
       </c>
       <c r="C177" t="n">
-        <v>24105.40565</v>
+        <v>289264.8678</v>
       </c>
     </row>
     <row r="178">
@@ -56804,7 +56804,7 @@
         <v>7</v>
       </c>
       <c r="C178" t="n">
-        <v>24105.40565</v>
+        <v>289264.8678</v>
       </c>
     </row>
     <row r="179">
@@ -56815,7 +56815,7 @@
         <v>8</v>
       </c>
       <c r="C179" t="n">
-        <v>24105.40565</v>
+        <v>289264.8678</v>
       </c>
     </row>
     <row r="180">
@@ -56826,7 +56826,7 @@
         <v>9</v>
       </c>
       <c r="C180" t="n">
-        <v>24105.40565</v>
+        <v>289264.8678</v>
       </c>
     </row>
     <row r="181">
@@ -56837,7 +56837,7 @@
         <v>10</v>
       </c>
       <c r="C181" t="n">
-        <v>24105.40565</v>
+        <v>289264.8678</v>
       </c>
     </row>
     <row r="182">
@@ -56848,7 +56848,7 @@
         <v>11</v>
       </c>
       <c r="C182" t="n">
-        <v>24105.40565</v>
+        <v>289264.8678</v>
       </c>
     </row>
     <row r="183">
@@ -56859,7 +56859,7 @@
         <v>12</v>
       </c>
       <c r="C183" t="n">
-        <v>24105.40565</v>
+        <v>289264.8678</v>
       </c>
     </row>
     <row r="184">
@@ -56881,7 +56881,7 @@
         <v>1</v>
       </c>
       <c r="C185" t="n">
-        <v>24510.5059</v>
+        <v>294126.0708</v>
       </c>
     </row>
     <row r="186">
@@ -56892,7 +56892,7 @@
         <v>2</v>
       </c>
       <c r="C186" t="n">
-        <v>24510.5059</v>
+        <v>294126.0708</v>
       </c>
     </row>
     <row r="187">
@@ -56903,7 +56903,7 @@
         <v>3</v>
       </c>
       <c r="C187" t="n">
-        <v>24510.5059</v>
+        <v>294126.0708</v>
       </c>
     </row>
     <row r="188">
@@ -56914,7 +56914,7 @@
         <v>4</v>
       </c>
       <c r="C188" t="n">
-        <v>24510.5059</v>
+        <v>294126.0708</v>
       </c>
     </row>
     <row r="189">
@@ -56925,7 +56925,7 @@
         <v>5</v>
       </c>
       <c r="C189" t="n">
-        <v>24510.5059</v>
+        <v>294126.0708</v>
       </c>
     </row>
     <row r="190">
@@ -56936,7 +56936,7 @@
         <v>6</v>
       </c>
       <c r="C190" t="n">
-        <v>24510.5059</v>
+        <v>294126.0708</v>
       </c>
     </row>
     <row r="191">
@@ -56947,7 +56947,7 @@
         <v>7</v>
       </c>
       <c r="C191" t="n">
-        <v>24510.5059</v>
+        <v>294126.0708</v>
       </c>
     </row>
     <row r="192">
@@ -56958,7 +56958,7 @@
         <v>8</v>
       </c>
       <c r="C192" t="n">
-        <v>24510.5059</v>
+        <v>294126.0708</v>
       </c>
     </row>
     <row r="193">
@@ -56969,7 +56969,7 @@
         <v>9</v>
       </c>
       <c r="C193" t="n">
-        <v>24510.5059</v>
+        <v>294126.0708</v>
       </c>
     </row>
     <row r="194">
@@ -56980,7 +56980,7 @@
         <v>10</v>
       </c>
       <c r="C194" t="n">
-        <v>24510.5059</v>
+        <v>294126.0708</v>
       </c>
     </row>
     <row r="195">
@@ -56991,7 +56991,7 @@
         <v>11</v>
       </c>
       <c r="C195" t="n">
-        <v>24510.5059</v>
+        <v>294126.0708</v>
       </c>
     </row>
     <row r="196">
@@ -57002,7 +57002,7 @@
         <v>12</v>
       </c>
       <c r="C196" t="n">
-        <v>24510.5059</v>
+        <v>294126.0708</v>
       </c>
     </row>
     <row r="197">
@@ -57024,7 +57024,7 @@
         <v>1</v>
       </c>
       <c r="C198" t="n">
-        <v>24915.60616666667</v>
+        <v>298987.274</v>
       </c>
     </row>
     <row r="199">
@@ -57035,7 +57035,7 @@
         <v>2</v>
       </c>
       <c r="C199" t="n">
-        <v>24915.60616666667</v>
+        <v>298987.274</v>
       </c>
     </row>
     <row r="200">
@@ -57046,7 +57046,7 @@
         <v>3</v>
       </c>
       <c r="C200" t="n">
-        <v>24915.60616666667</v>
+        <v>298987.274</v>
       </c>
     </row>
     <row r="201">
@@ -57057,7 +57057,7 @@
         <v>4</v>
       </c>
       <c r="C201" t="n">
-        <v>24915.60616666667</v>
+        <v>298987.274</v>
       </c>
     </row>
     <row r="202">
@@ -57068,7 +57068,7 @@
         <v>5</v>
       </c>
       <c r="C202" t="n">
-        <v>24915.60616666667</v>
+        <v>298987.274</v>
       </c>
     </row>
     <row r="203">
@@ -57079,7 +57079,7 @@
         <v>6</v>
       </c>
       <c r="C203" t="n">
-        <v>24915.60616666667</v>
+        <v>298987.274</v>
       </c>
     </row>
     <row r="204">
@@ -57090,7 +57090,7 @@
         <v>7</v>
       </c>
       <c r="C204" t="n">
-        <v>24915.60616666667</v>
+        <v>298987.274</v>
       </c>
     </row>
     <row r="205">
@@ -57101,7 +57101,7 @@
         <v>8</v>
       </c>
       <c r="C205" t="n">
-        <v>24915.60616666667</v>
+        <v>298987.274</v>
       </c>
     </row>
     <row r="206">
@@ -57112,7 +57112,7 @@
         <v>9</v>
       </c>
       <c r="C206" t="n">
-        <v>24915.60616666667</v>
+        <v>298987.274</v>
       </c>
     </row>
     <row r="207">
@@ -57123,7 +57123,7 @@
         <v>10</v>
       </c>
       <c r="C207" t="n">
-        <v>24915.60616666667</v>
+        <v>298987.274</v>
       </c>
     </row>
     <row r="208">
@@ -57134,7 +57134,7 @@
         <v>11</v>
       </c>
       <c r="C208" t="n">
-        <v>24915.60616666667</v>
+        <v>298987.274</v>
       </c>
     </row>
     <row r="209">
@@ -57145,7 +57145,7 @@
         <v>12</v>
       </c>
       <c r="C209" t="n">
-        <v>24915.60616666667</v>
+        <v>298987.274</v>
       </c>
     </row>
     <row r="210">
@@ -57167,7 +57167,7 @@
         <v>1</v>
       </c>
       <c r="C211" t="n">
-        <v>24544.503775</v>
+        <v>294534.0453</v>
       </c>
     </row>
     <row r="212">
@@ -57178,7 +57178,7 @@
         <v>2</v>
       </c>
       <c r="C212" t="n">
-        <v>24544.503775</v>
+        <v>294534.0453</v>
       </c>
     </row>
     <row r="213">
@@ -57189,7 +57189,7 @@
         <v>3</v>
       </c>
       <c r="C213" t="n">
-        <v>24544.503775</v>
+        <v>294534.0453</v>
       </c>
     </row>
     <row r="214">
@@ -57200,7 +57200,7 @@
         <v>4</v>
       </c>
       <c r="C214" t="n">
-        <v>24544.503775</v>
+        <v>294534.0453</v>
       </c>
     </row>
     <row r="215">
@@ -57211,7 +57211,7 @@
         <v>5</v>
       </c>
       <c r="C215" t="n">
-        <v>24544.503775</v>
+        <v>294534.0453</v>
       </c>
     </row>
     <row r="216">
@@ -57222,7 +57222,7 @@
         <v>6</v>
       </c>
       <c r="C216" t="n">
-        <v>24544.503775</v>
+        <v>294534.0453</v>
       </c>
     </row>
     <row r="217">
@@ -57233,7 +57233,7 @@
         <v>7</v>
       </c>
       <c r="C217" t="n">
-        <v>24544.503775</v>
+        <v>294534.0453</v>
       </c>
     </row>
     <row r="218">
@@ -57244,7 +57244,7 @@
         <v>8</v>
       </c>
       <c r="C218" t="n">
-        <v>24544.503775</v>
+        <v>294534.0453</v>
       </c>
     </row>
     <row r="219">
@@ -57255,7 +57255,7 @@
         <v>9</v>
       </c>
       <c r="C219" t="n">
-        <v>24544.503775</v>
+        <v>294534.0453</v>
       </c>
     </row>
     <row r="220">
@@ -57266,7 +57266,7 @@
         <v>10</v>
       </c>
       <c r="C220" t="n">
-        <v>24544.503775</v>
+        <v>294534.0453</v>
       </c>
     </row>
     <row r="221">
@@ -57277,7 +57277,7 @@
         <v>11</v>
       </c>
       <c r="C221" t="n">
-        <v>24544.503775</v>
+        <v>294534.0453</v>
       </c>
     </row>
     <row r="222">
@@ -57288,7 +57288,7 @@
         <v>12</v>
       </c>
       <c r="C222" t="n">
-        <v>24544.503775</v>
+        <v>294534.0453</v>
       </c>
     </row>
     <row r="223">
@@ -57310,7 +57310,7 @@
         <v>1</v>
       </c>
       <c r="C224" t="n">
-        <v>24894.55395</v>
+        <v>298734.6474</v>
       </c>
     </row>
     <row r="225">
@@ -57321,7 +57321,7 @@
         <v>2</v>
       </c>
       <c r="C225" t="n">
-        <v>24894.55395</v>
+        <v>298734.6474</v>
       </c>
     </row>
     <row r="226">
@@ -57332,7 +57332,7 @@
         <v>3</v>
       </c>
       <c r="C226" t="n">
-        <v>24894.55395</v>
+        <v>298734.6474</v>
       </c>
     </row>
     <row r="227">
@@ -57343,7 +57343,7 @@
         <v>4</v>
       </c>
       <c r="C227" t="n">
-        <v>24894.55395</v>
+        <v>298734.6474</v>
       </c>
     </row>
     <row r="228">
@@ -57354,7 +57354,7 @@
         <v>5</v>
       </c>
       <c r="C228" t="n">
-        <v>24894.55395</v>
+        <v>298734.6474</v>
       </c>
     </row>
     <row r="229">
@@ -57365,7 +57365,7 @@
         <v>6</v>
       </c>
       <c r="C229" t="n">
-        <v>24894.55395</v>
+        <v>298734.6474</v>
       </c>
     </row>
     <row r="230">
@@ -57376,7 +57376,7 @@
         <v>7</v>
       </c>
       <c r="C230" t="n">
-        <v>24894.55395</v>
+        <v>298734.6474</v>
       </c>
     </row>
     <row r="231">
@@ -57387,7 +57387,7 @@
         <v>8</v>
       </c>
       <c r="C231" t="n">
-        <v>24894.55395</v>
+        <v>298734.6474</v>
       </c>
     </row>
     <row r="232">
@@ -57398,7 +57398,7 @@
         <v>9</v>
       </c>
       <c r="C232" t="n">
-        <v>24894.55395</v>
+        <v>298734.6474</v>
       </c>
     </row>
     <row r="233">
@@ -57409,7 +57409,7 @@
         <v>10</v>
       </c>
       <c r="C233" t="n">
-        <v>24894.55395</v>
+        <v>298734.6474</v>
       </c>
     </row>
     <row r="234">
@@ -57420,7 +57420,7 @@
         <v>11</v>
       </c>
       <c r="C234" t="n">
-        <v>24894.55395</v>
+        <v>298734.6474</v>
       </c>
     </row>
     <row r="235">
@@ -57431,7 +57431,7 @@
         <v>12</v>
       </c>
       <c r="C235" t="n">
-        <v>24894.55395</v>
+        <v>298734.6474</v>
       </c>
     </row>
     <row r="236">
@@ -57453,7 +57453,7 @@
         <v>1</v>
       </c>
       <c r="C237" t="n">
-        <v>25244.60413333334</v>
+        <v>302935.2496</v>
       </c>
     </row>
     <row r="238">
@@ -57464,7 +57464,7 @@
         <v>2</v>
       </c>
       <c r="C238" t="n">
-        <v>25244.60413333334</v>
+        <v>302935.2496</v>
       </c>
     </row>
     <row r="239">
@@ -57475,7 +57475,7 @@
         <v>3</v>
       </c>
       <c r="C239" t="n">
-        <v>25244.60413333334</v>
+        <v>302935.2496</v>
       </c>
     </row>
     <row r="240">
@@ -57486,7 +57486,7 @@
         <v>4</v>
       </c>
       <c r="C240" t="n">
-        <v>25244.60413333334</v>
+        <v>302935.2496</v>
       </c>
     </row>
     <row r="241">
@@ -57497,7 +57497,7 @@
         <v>5</v>
       </c>
       <c r="C241" t="n">
-        <v>25244.60413333334</v>
+        <v>302935.2496</v>
       </c>
     </row>
     <row r="242">
@@ -57508,7 +57508,7 @@
         <v>6</v>
       </c>
       <c r="C242" t="n">
-        <v>25244.60413333334</v>
+        <v>302935.2496</v>
       </c>
     </row>
     <row r="243">
@@ -57519,7 +57519,7 @@
         <v>7</v>
       </c>
       <c r="C243" t="n">
-        <v>25244.60413333334</v>
+        <v>302935.2496</v>
       </c>
     </row>
     <row r="244">
@@ -57530,7 +57530,7 @@
         <v>8</v>
       </c>
       <c r="C244" t="n">
-        <v>25244.60413333334</v>
+        <v>302935.2496</v>
       </c>
     </row>
     <row r="245">
@@ -57541,7 +57541,7 @@
         <v>9</v>
       </c>
       <c r="C245" t="n">
-        <v>25244.60413333334</v>
+        <v>302935.2496</v>
       </c>
     </row>
     <row r="246">
@@ -57552,7 +57552,7 @@
         <v>10</v>
       </c>
       <c r="C246" t="n">
-        <v>25244.60413333334</v>
+        <v>302935.2496</v>
       </c>
     </row>
     <row r="247">
@@ -57563,7 +57563,7 @@
         <v>11</v>
       </c>
       <c r="C247" t="n">
-        <v>25244.60413333334</v>
+        <v>302935.2496</v>
       </c>
     </row>
     <row r="248">
@@ -57574,7 +57574,7 @@
         <v>12</v>
       </c>
       <c r="C248" t="n">
-        <v>25244.60413333334</v>
+        <v>302935.2496</v>
       </c>
     </row>
     <row r="249">
@@ -57596,7 +57596,7 @@
         <v>1</v>
       </c>
       <c r="C250" t="n">
-        <v>25594.65430833333</v>
+        <v>307135.8517</v>
       </c>
     </row>
     <row r="251">
@@ -57607,7 +57607,7 @@
         <v>2</v>
       </c>
       <c r="C251" t="n">
-        <v>25594.65430833333</v>
+        <v>307135.8517</v>
       </c>
     </row>
     <row r="252">
@@ -57618,7 +57618,7 @@
         <v>3</v>
       </c>
       <c r="C252" t="n">
-        <v>25594.65430833333</v>
+        <v>307135.8517</v>
       </c>
     </row>
     <row r="253">
@@ -57629,7 +57629,7 @@
         <v>4</v>
       </c>
       <c r="C253" t="n">
-        <v>25594.65430833333</v>
+        <v>307135.8517</v>
       </c>
     </row>
     <row r="254">
@@ -57640,7 +57640,7 @@
         <v>5</v>
       </c>
       <c r="C254" t="n">
-        <v>25594.65430833333</v>
+        <v>307135.8517</v>
       </c>
     </row>
     <row r="255">
@@ -57651,7 +57651,7 @@
         <v>6</v>
       </c>
       <c r="C255" t="n">
-        <v>25594.65430833333</v>
+        <v>307135.8517</v>
       </c>
     </row>
     <row r="256">
@@ -57662,7 +57662,7 @@
         <v>7</v>
       </c>
       <c r="C256" t="n">
-        <v>25594.65430833333</v>
+        <v>307135.8517</v>
       </c>
     </row>
     <row r="257">
@@ -57673,7 +57673,7 @@
         <v>8</v>
       </c>
       <c r="C257" t="n">
-        <v>25594.65430833333</v>
+        <v>307135.8517</v>
       </c>
     </row>
     <row r="258">
@@ -57684,7 +57684,7 @@
         <v>9</v>
       </c>
       <c r="C258" t="n">
-        <v>25594.65430833333</v>
+        <v>307135.8517</v>
       </c>
     </row>
     <row r="259">
@@ -57695,7 +57695,7 @@
         <v>10</v>
       </c>
       <c r="C259" t="n">
-        <v>25594.65430833333</v>
+        <v>307135.8517</v>
       </c>
     </row>
     <row r="260">
@@ -57706,7 +57706,7 @@
         <v>11</v>
       </c>
       <c r="C260" t="n">
-        <v>25594.65430833333</v>
+        <v>307135.8517</v>
       </c>
     </row>
     <row r="261">
@@ -57717,7 +57717,7 @@
         <v>12</v>
       </c>
       <c r="C261" t="n">
-        <v>25594.65430833333</v>
+        <v>307135.8517</v>
       </c>
     </row>
     <row r="262">
@@ -57739,7 +57739,7 @@
         <v>1</v>
       </c>
       <c r="C263" t="n">
-        <v>25944.70448333333</v>
+        <v>311336.4538</v>
       </c>
     </row>
     <row r="264">
@@ -57750,7 +57750,7 @@
         <v>2</v>
       </c>
       <c r="C264" t="n">
-        <v>25944.70448333333</v>
+        <v>311336.4538</v>
       </c>
     </row>
     <row r="265">
@@ -57761,7 +57761,7 @@
         <v>3</v>
       </c>
       <c r="C265" t="n">
-        <v>25944.70448333333</v>
+        <v>311336.4538</v>
       </c>
     </row>
     <row r="266">
@@ -57772,7 +57772,7 @@
         <v>4</v>
       </c>
       <c r="C266" t="n">
-        <v>25944.70448333333</v>
+        <v>311336.4538</v>
       </c>
     </row>
     <row r="267">
@@ -57783,7 +57783,7 @@
         <v>5</v>
       </c>
       <c r="C267" t="n">
-        <v>25944.70448333333</v>
+        <v>311336.4538</v>
       </c>
     </row>
     <row r="268">
@@ -57794,7 +57794,7 @@
         <v>6</v>
       </c>
       <c r="C268" t="n">
-        <v>25944.70448333333</v>
+        <v>311336.4538</v>
       </c>
     </row>
     <row r="269">
@@ -57805,7 +57805,7 @@
         <v>7</v>
       </c>
       <c r="C269" t="n">
-        <v>25944.70448333333</v>
+        <v>311336.4538</v>
       </c>
     </row>
     <row r="270">
@@ -57816,7 +57816,7 @@
         <v>8</v>
       </c>
       <c r="C270" t="n">
-        <v>25944.70448333333</v>
+        <v>311336.4538</v>
       </c>
     </row>
     <row r="271">
@@ -57827,7 +57827,7 @@
         <v>9</v>
       </c>
       <c r="C271" t="n">
-        <v>25944.70448333333</v>
+        <v>311336.4538</v>
       </c>
     </row>
     <row r="272">
@@ -57838,7 +57838,7 @@
         <v>10</v>
       </c>
       <c r="C272" t="n">
-        <v>25944.70448333333</v>
+        <v>311336.4538</v>
       </c>
     </row>
     <row r="273">
@@ -57849,7 +57849,7 @@
         <v>11</v>
       </c>
       <c r="C273" t="n">
-        <v>25944.70448333333</v>
+        <v>311336.4538</v>
       </c>
     </row>
     <row r="274">
@@ -57860,7 +57860,7 @@
         <v>12</v>
       </c>
       <c r="C274" t="n">
-        <v>25944.70448333333</v>
+        <v>311336.4538</v>
       </c>
     </row>
     <row r="275">
@@ -57882,7 +57882,7 @@
         <v>1</v>
       </c>
       <c r="C276" t="n">
-        <v>26294.75465833333</v>
+        <v>315537.0559</v>
       </c>
     </row>
     <row r="277">
@@ -57893,7 +57893,7 @@
         <v>2</v>
       </c>
       <c r="C277" t="n">
-        <v>26294.75465833333</v>
+        <v>315537.0559</v>
       </c>
     </row>
     <row r="278">
@@ -57904,7 +57904,7 @@
         <v>3</v>
       </c>
       <c r="C278" t="n">
-        <v>26294.75465833333</v>
+        <v>315537.0559</v>
       </c>
     </row>
     <row r="279">
@@ -57915,7 +57915,7 @@
         <v>4</v>
       </c>
       <c r="C279" t="n">
-        <v>26294.75465833333</v>
+        <v>315537.0559</v>
       </c>
     </row>
     <row r="280">
@@ -57926,7 +57926,7 @@
         <v>5</v>
       </c>
       <c r="C280" t="n">
-        <v>26294.75465833333</v>
+        <v>315537.0559</v>
       </c>
     </row>
     <row r="281">
@@ -57937,7 +57937,7 @@
         <v>6</v>
       </c>
       <c r="C281" t="n">
-        <v>26294.75465833333</v>
+        <v>315537.0559</v>
       </c>
     </row>
     <row r="282">
@@ -57948,7 +57948,7 @@
         <v>7</v>
       </c>
       <c r="C282" t="n">
-        <v>26294.75465833333</v>
+        <v>315537.0559</v>
       </c>
     </row>
     <row r="283">
@@ -57959,7 +57959,7 @@
         <v>8</v>
       </c>
       <c r="C283" t="n">
-        <v>26294.75465833333</v>
+        <v>315537.0559</v>
       </c>
     </row>
     <row r="284">
@@ -57970,7 +57970,7 @@
         <v>9</v>
       </c>
       <c r="C284" t="n">
-        <v>26294.75465833333</v>
+        <v>315537.0559</v>
       </c>
     </row>
     <row r="285">
@@ -57981,7 +57981,7 @@
         <v>10</v>
       </c>
       <c r="C285" t="n">
-        <v>26294.75465833333</v>
+        <v>315537.0559</v>
       </c>
     </row>
     <row r="286">
@@ -57992,7 +57992,7 @@
         <v>11</v>
       </c>
       <c r="C286" t="n">
-        <v>26294.75465833333</v>
+        <v>315537.0559</v>
       </c>
     </row>
     <row r="287">
@@ -58003,7 +58003,7 @@
         <v>12</v>
       </c>
       <c r="C287" t="n">
-        <v>26294.75465833333</v>
+        <v>315537.0559</v>
       </c>
     </row>
     <row r="288">
@@ -58025,7 +58025,7 @@
         <v>1</v>
       </c>
       <c r="C289" t="n">
-        <v>26644.80484166667</v>
+        <v>319737.6581000001</v>
       </c>
     </row>
     <row r="290">
@@ -58036,7 +58036,7 @@
         <v>2</v>
       </c>
       <c r="C290" t="n">
-        <v>26644.80484166667</v>
+        <v>319737.6581000001</v>
       </c>
     </row>
     <row r="291">
@@ -58047,7 +58047,7 @@
         <v>3</v>
       </c>
       <c r="C291" t="n">
-        <v>26644.80484166667</v>
+        <v>319737.6581000001</v>
       </c>
     </row>
     <row r="292">
@@ -58058,7 +58058,7 @@
         <v>4</v>
       </c>
       <c r="C292" t="n">
-        <v>26644.80484166667</v>
+        <v>319737.6581000001</v>
       </c>
     </row>
     <row r="293">
@@ -58069,7 +58069,7 @@
         <v>5</v>
       </c>
       <c r="C293" t="n">
-        <v>26644.80484166667</v>
+        <v>319737.6581000001</v>
       </c>
     </row>
     <row r="294">
@@ -58080,7 +58080,7 @@
         <v>6</v>
       </c>
       <c r="C294" t="n">
-        <v>26644.80484166667</v>
+        <v>319737.6581000001</v>
       </c>
     </row>
     <row r="295">
@@ -58091,7 +58091,7 @@
         <v>7</v>
       </c>
       <c r="C295" t="n">
-        <v>26644.80484166667</v>
+        <v>319737.6581000001</v>
       </c>
     </row>
     <row r="296">
@@ -58102,7 +58102,7 @@
         <v>8</v>
       </c>
       <c r="C296" t="n">
-        <v>26644.80484166667</v>
+        <v>319737.6581000001</v>
       </c>
     </row>
     <row r="297">
@@ -58113,7 +58113,7 @@
         <v>9</v>
       </c>
       <c r="C297" t="n">
-        <v>26644.80484166667</v>
+        <v>319737.6581000001</v>
       </c>
     </row>
     <row r="298">
@@ -58124,7 +58124,7 @@
         <v>10</v>
       </c>
       <c r="C298" t="n">
-        <v>26644.80484166667</v>
+        <v>319737.6581000001</v>
       </c>
     </row>
     <row r="299">
@@ -58135,7 +58135,7 @@
         <v>11</v>
       </c>
       <c r="C299" t="n">
-        <v>26644.80484166667</v>
+        <v>319737.6581000001</v>
       </c>
     </row>
     <row r="300">
@@ -58146,7 +58146,7 @@
         <v>12</v>
       </c>
       <c r="C300" t="n">
-        <v>26644.80484166667</v>
+        <v>319737.6581000001</v>
       </c>
     </row>
     <row r="301">
@@ -58168,7 +58168,7 @@
         <v>1</v>
       </c>
       <c r="C302" t="n">
-        <v>26994.85501666667</v>
+        <v>323938.2602</v>
       </c>
     </row>
     <row r="303">
@@ -58179,7 +58179,7 @@
         <v>2</v>
       </c>
       <c r="C303" t="n">
-        <v>26994.85501666667</v>
+        <v>323938.2602</v>
       </c>
     </row>
     <row r="304">
@@ -58190,7 +58190,7 @@
         <v>3</v>
       </c>
       <c r="C304" t="n">
-        <v>26994.85501666667</v>
+        <v>323938.2602</v>
       </c>
     </row>
     <row r="305">
@@ -58201,7 +58201,7 @@
         <v>4</v>
       </c>
       <c r="C305" t="n">
-        <v>26994.85501666667</v>
+        <v>323938.2602</v>
       </c>
     </row>
     <row r="306">
@@ -58212,7 +58212,7 @@
         <v>5</v>
       </c>
       <c r="C306" t="n">
-        <v>26994.85501666667</v>
+        <v>323938.2602</v>
       </c>
     </row>
     <row r="307">
@@ -58223,7 +58223,7 @@
         <v>6</v>
       </c>
       <c r="C307" t="n">
-        <v>26994.85501666667</v>
+        <v>323938.2602</v>
       </c>
     </row>
     <row r="308">
@@ -58234,7 +58234,7 @@
         <v>7</v>
       </c>
       <c r="C308" t="n">
-        <v>26994.85501666667</v>
+        <v>323938.2602</v>
       </c>
     </row>
     <row r="309">
@@ -58245,7 +58245,7 @@
         <v>8</v>
       </c>
       <c r="C309" t="n">
-        <v>26994.85501666667</v>
+        <v>323938.2602</v>
       </c>
     </row>
     <row r="310">
@@ -58256,7 +58256,7 @@
         <v>9</v>
       </c>
       <c r="C310" t="n">
-        <v>26994.85501666667</v>
+        <v>323938.2602</v>
       </c>
     </row>
     <row r="311">
@@ -58267,7 +58267,7 @@
         <v>10</v>
       </c>
       <c r="C311" t="n">
-        <v>26994.85501666667</v>
+        <v>323938.2602</v>
       </c>
     </row>
     <row r="312">
@@ -58278,7 +58278,7 @@
         <v>11</v>
       </c>
       <c r="C312" t="n">
-        <v>26994.85501666667</v>
+        <v>323938.2602</v>
       </c>
     </row>
     <row r="313">
@@ -58289,7 +58289,7 @@
         <v>12</v>
       </c>
       <c r="C313" t="n">
-        <v>26994.85501666667</v>
+        <v>323938.2602</v>
       </c>
     </row>
     <row r="314">
@@ -58311,7 +58311,7 @@
         <v>1</v>
       </c>
       <c r="C315" t="n">
-        <v>27344.90519166667</v>
+        <v>328138.8623</v>
       </c>
     </row>
     <row r="316">
@@ -58322,7 +58322,7 @@
         <v>2</v>
       </c>
       <c r="C316" t="n">
-        <v>27344.90519166667</v>
+        <v>328138.8623</v>
       </c>
     </row>
     <row r="317">
@@ -58333,7 +58333,7 @@
         <v>3</v>
       </c>
       <c r="C317" t="n">
-        <v>27344.90519166667</v>
+        <v>328138.8623</v>
       </c>
     </row>
     <row r="318">
@@ -58344,7 +58344,7 @@
         <v>4</v>
       </c>
       <c r="C318" t="n">
-        <v>27344.90519166667</v>
+        <v>328138.8623</v>
       </c>
     </row>
     <row r="319">
@@ -58355,7 +58355,7 @@
         <v>5</v>
       </c>
       <c r="C319" t="n">
-        <v>27344.90519166667</v>
+        <v>328138.8623</v>
       </c>
     </row>
     <row r="320">
@@ -58366,7 +58366,7 @@
         <v>6</v>
       </c>
       <c r="C320" t="n">
-        <v>27344.90519166667</v>
+        <v>328138.8623</v>
       </c>
     </row>
     <row r="321">
@@ -58377,7 +58377,7 @@
         <v>7</v>
       </c>
       <c r="C321" t="n">
-        <v>27344.90519166667</v>
+        <v>328138.8623</v>
       </c>
     </row>
     <row r="322">
@@ -58388,7 +58388,7 @@
         <v>8</v>
       </c>
       <c r="C322" t="n">
-        <v>27344.90519166667</v>
+        <v>328138.8623</v>
       </c>
     </row>
     <row r="323">
@@ -58399,7 +58399,7 @@
         <v>9</v>
       </c>
       <c r="C323" t="n">
-        <v>27344.90519166667</v>
+        <v>328138.8623</v>
       </c>
     </row>
     <row r="324">
@@ -58410,7 +58410,7 @@
         <v>10</v>
       </c>
       <c r="C324" t="n">
-        <v>27344.90519166667</v>
+        <v>328138.8623</v>
       </c>
     </row>
     <row r="325">
@@ -58421,7 +58421,7 @@
         <v>11</v>
       </c>
       <c r="C325" t="n">
-        <v>27344.90519166667</v>
+        <v>328138.8623</v>
       </c>
     </row>
     <row r="326">
@@ -58432,7 +58432,7 @@
         <v>12</v>
       </c>
       <c r="C326" t="n">
-        <v>27344.90519166667</v>
+        <v>328138.8623</v>
       </c>
     </row>
     <row r="327">
@@ -58454,7 +58454,7 @@
         <v>1</v>
       </c>
       <c r="C328" t="n">
-        <v>27694.95536666667</v>
+        <v>332339.4644</v>
       </c>
     </row>
     <row r="329">
@@ -58465,7 +58465,7 @@
         <v>2</v>
       </c>
       <c r="C329" t="n">
-        <v>27694.95536666667</v>
+        <v>332339.4644</v>
       </c>
     </row>
     <row r="330">
@@ -58476,7 +58476,7 @@
         <v>3</v>
       </c>
       <c r="C330" t="n">
-        <v>27694.95536666667</v>
+        <v>332339.4644</v>
       </c>
     </row>
     <row r="331">
@@ -58487,7 +58487,7 @@
         <v>4</v>
       </c>
       <c r="C331" t="n">
-        <v>27694.95536666667</v>
+        <v>332339.4644</v>
       </c>
     </row>
     <row r="332">
@@ -58498,7 +58498,7 @@
         <v>5</v>
       </c>
       <c r="C332" t="n">
-        <v>27694.95536666667</v>
+        <v>332339.4644</v>
       </c>
     </row>
     <row r="333">
@@ -58509,7 +58509,7 @@
         <v>6</v>
       </c>
       <c r="C333" t="n">
-        <v>27694.95536666667</v>
+        <v>332339.4644</v>
       </c>
     </row>
     <row r="334">
@@ -58520,7 +58520,7 @@
         <v>7</v>
       </c>
       <c r="C334" t="n">
-        <v>27694.95536666667</v>
+        <v>332339.4644</v>
       </c>
     </row>
     <row r="335">
@@ -58531,7 +58531,7 @@
         <v>8</v>
       </c>
       <c r="C335" t="n">
-        <v>27694.95536666667</v>
+        <v>332339.4644</v>
       </c>
     </row>
     <row r="336">
@@ -58542,7 +58542,7 @@
         <v>9</v>
       </c>
       <c r="C336" t="n">
-        <v>27694.95536666667</v>
+        <v>332339.4644</v>
       </c>
     </row>
     <row r="337">
@@ -58553,7 +58553,7 @@
         <v>10</v>
       </c>
       <c r="C337" t="n">
-        <v>27694.95536666667</v>
+        <v>332339.4644</v>
       </c>
     </row>
     <row r="338">
@@ -58564,7 +58564,7 @@
         <v>11</v>
       </c>
       <c r="C338" t="n">
-        <v>27694.95536666667</v>
+        <v>332339.4644</v>
       </c>
     </row>
     <row r="339">
@@ -58575,7 +58575,7 @@
         <v>12</v>
       </c>
       <c r="C339" t="n">
-        <v>27694.95536666667</v>
+        <v>332339.4644</v>
       </c>
     </row>
     <row r="340">
@@ -58597,7 +58597,7 @@
         <v>1</v>
       </c>
       <c r="C341" t="n">
-        <v>28215.06606666667</v>
+        <v>338580.7928</v>
       </c>
     </row>
     <row r="342">
@@ -58608,7 +58608,7 @@
         <v>2</v>
       </c>
       <c r="C342" t="n">
-        <v>28215.06606666667</v>
+        <v>338580.7928</v>
       </c>
     </row>
     <row r="343">
@@ -58619,7 +58619,7 @@
         <v>3</v>
       </c>
       <c r="C343" t="n">
-        <v>28215.06606666667</v>
+        <v>338580.7928</v>
       </c>
     </row>
     <row r="344">
@@ -58630,7 +58630,7 @@
         <v>4</v>
       </c>
       <c r="C344" t="n">
-        <v>28215.06606666667</v>
+        <v>338580.7928</v>
       </c>
     </row>
     <row r="345">
@@ -58641,7 +58641,7 @@
         <v>5</v>
       </c>
       <c r="C345" t="n">
-        <v>28215.06606666667</v>
+        <v>338580.7928</v>
       </c>
     </row>
     <row r="346">
@@ -58652,7 +58652,7 @@
         <v>6</v>
       </c>
       <c r="C346" t="n">
-        <v>28215.06606666667</v>
+        <v>338580.7928</v>
       </c>
     </row>
     <row r="347">
@@ -58663,7 +58663,7 @@
         <v>7</v>
       </c>
       <c r="C347" t="n">
-        <v>28215.06606666667</v>
+        <v>338580.7928</v>
       </c>
     </row>
     <row r="348">
@@ -58674,7 +58674,7 @@
         <v>8</v>
       </c>
       <c r="C348" t="n">
-        <v>28215.06606666667</v>
+        <v>338580.7928</v>
       </c>
     </row>
     <row r="349">
@@ -58685,7 +58685,7 @@
         <v>9</v>
       </c>
       <c r="C349" t="n">
-        <v>28215.06606666667</v>
+        <v>338580.7928</v>
       </c>
     </row>
     <row r="350">
@@ -58696,7 +58696,7 @@
         <v>10</v>
       </c>
       <c r="C350" t="n">
-        <v>28215.06606666667</v>
+        <v>338580.7928</v>
       </c>
     </row>
     <row r="351">
@@ -58707,7 +58707,7 @@
         <v>11</v>
       </c>
       <c r="C351" t="n">
-        <v>28215.06606666667</v>
+        <v>338580.7928</v>
       </c>
     </row>
     <row r="352">
@@ -58718,7 +58718,7 @@
         <v>12</v>
       </c>
       <c r="C352" t="n">
-        <v>28215.06606666667</v>
+        <v>338580.7928</v>
       </c>
     </row>
   </sheetData>

</xml_diff>